<commit_message>
Docker em um comando, preços finais e polimento do CRM
- Dockerfile multi-etapas (build do frontend embutido na API) e compose com
  MySQL 8 (fuso -03:00, healthcheck) + app; `docker compose up -d --build`
  sobe tudo em http://localhost:3040; .env.example na raiz de foro_app
- Preços: Starter R$ 129,90 / Pro R$ 199,90 / Business R$ 399,90; consultas
  por semana 5/10/15/20 (trial/starter/pro/business); docs e planilha atualizadas
- Frontend: detalhe do lead editável com tarefas e notas, Tarefas agrupadas
  (atrasadas/hoje/próximas) com check, Painel com funil colorido e créditos,
  página de planos com valores em centavos e selo "Mais escolhido"

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GyobEssboDTUuesieuqap
</commit_message>
<xml_diff>
--- a/foro_app/documentation/precificacao_foro_semanal.xlsx
+++ b/foro_app/documentation/precificacao_foro_semanal.xlsx
@@ -585,13 +585,13 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>97</v>
+        <v>129.9</v>
       </c>
       <c r="D2" t="n">
-        <v>197</v>
+        <v>199.9</v>
       </c>
       <c r="E2" t="n">
-        <v>397</v>
+        <v>399.9</v>
       </c>
     </row>
     <row r="3">
@@ -639,13 +639,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E5" t="n">
         <v>20</v>

</xml_diff>